<commit_message>
updated readme, fixed minor issues in Stage_2.
</commit_message>
<xml_diff>
--- a/Stage_2/5_spatial_information/spatial_information_plot.xlsx
+++ b/Stage_2/5_spatial_information/spatial_information_plot.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IUcodings\Protocol_speech_recog\github_clean\procedure_2\5_spatial_information\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IUcodings\Protocol_speech_recog\github_clean\Stage_2\5_spatial_information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39B4F8C5-6D96-47A0-9531-B87AF2275D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C795096E-C0F7-486C-A921-1E5E6E4FC57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{04C333F3-0F63-4974-A2A0-69290A084773}"/>
   </bookViews>
   <sheets>
-    <sheet name="Fig 2e" sheetId="1" r:id="rId1"/>
+    <sheet name="Fig 3e" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>